<commit_message>
PAUSED (task161): stage 4 round 1 fixed in one rebuild, waiting on the re-judge
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A6XcFx5t62c7gPi1bBKcVi
</commit_message>
<xml_diff>
--- a/task161/golden/overflow_blocks_h1_2027.xlsx
+++ b/task161/golden/overflow_blocks_h1_2027.xlsx
@@ -9,9 +9,8 @@
   <sheets>
     <sheet name="Blocks" sheetId="1" r:id="rId1"/>
     <sheet name="By account" sheetId="2" r:id="rId2"/>
-    <sheet name="Off-rack 6 Dec" sheetId="3" r:id="rId3"/>
-    <sheet name="Port TEU 2026" sheetId="4" r:id="rId4"/>
-    <sheet name="Notes" sheetId="5" r:id="rId5"/>
+    <sheet name="Port TEU 2026" sheetId="3" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -23,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="123">
-  <si>
-    <t>Tamarind Avenue Logistics Park, Building B: the second block would be 97% used over January to June 2027, the third 10%</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="108">
+  <si>
+    <t>Tamarind Avenue Logistics Park, Building B: the second block would be 100% used over January to June 2027, the third 18%</t>
   </si>
   <si>
     <t>Capacity planning | forecast from the close of Sunday 6 December 2026 | prepared Monday 7 December 2026</t>
@@ -118,7 +117,7 @@
     <t>Monthly figures are rounded separately; the term totals and uses are computed before rounding. Notes: see the Notes sheet.</t>
   </si>
   <si>
-    <t>Five seasonal accounts hold 17,541 of the 20,063 pallets over normal stock at 31 December; 10,123 are still here at 30 June</t>
+    <t>Five seasonal accounts hold 18,511 of the 20,166 pallets over normal stock at 31 December; 11,826 are still here at 30 June</t>
   </si>
   <si>
     <t>Each account's excess over its normal stock leaves at the share of its own shipments its excess left at after the duty steps of 1 September 2019, 5 April 2025 and 7 August 2025, until it is gone.</t>
@@ -236,51 +235,6 @@
   </si>
   <si>
     <t>All accounts</t>
-  </si>
-  <si>
-    <t>Pallets outside our racks at the close of Sunday 6 December 2026, by building</t>
-  </si>
-  <si>
-    <t>On hand: nightly inventory run of 7 December 08:00Z. In racks: rack positions holding a pallet in the LPN export of the same run. Outside the racks: floor lanes, dock staging and storage trailers in the yard.</t>
-  </si>
-  <si>
-    <t>Building</t>
-  </si>
-  <si>
-    <t>Site</t>
-  </si>
-  <si>
-    <t>Pallets on hand</t>
-  </si>
-  <si>
-    <t>In rack positions</t>
-  </si>
-  <si>
-    <t>Outside the racks</t>
-  </si>
-  <si>
-    <t>Del Amo, Carson</t>
-  </si>
-  <si>
-    <t>CAR1</t>
-  </si>
-  <si>
-    <t>Alondra, Rancho Dominguez</t>
-  </si>
-  <si>
-    <t>RDZ1</t>
-  </si>
-  <si>
-    <t>Anaheim Street, Wilmington</t>
-  </si>
-  <si>
-    <t>WIL1</t>
-  </si>
-  <si>
-    <t>Artesia, Compton</t>
-  </si>
-  <si>
-    <t>CMP1</t>
   </si>
   <si>
     <t>Import containers whose freight reached us from the two ports, January to October 2026</t>
@@ -841,10 +795,10 @@
         <v>10</v>
       </c>
       <c r="B8" s="4">
-        <v>49294</v>
+        <v>48773</v>
       </c>
       <c r="C8" s="4">
-        <v>9294</v>
+        <v>8773</v>
       </c>
       <c r="D8" s="4">
         <v>4000</v>
@@ -853,7 +807,7 @@
         <v>4000</v>
       </c>
       <c r="F8" s="4">
-        <v>1294</v>
+        <v>773</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -861,10 +815,10 @@
         <v>11</v>
       </c>
       <c r="B9" s="4">
-        <v>48203</v>
+        <v>48063</v>
       </c>
       <c r="C9" s="4">
-        <v>8203</v>
+        <v>8063</v>
       </c>
       <c r="D9" s="4">
         <v>4000</v>
@@ -873,7 +827,7 @@
         <v>4000</v>
       </c>
       <c r="F9" s="4">
-        <v>203</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -881,10 +835,10 @@
         <v>12</v>
       </c>
       <c r="B10" s="4">
-        <v>48520</v>
+        <v>48786</v>
       </c>
       <c r="C10" s="4">
-        <v>8520</v>
+        <v>8786</v>
       </c>
       <c r="D10" s="4">
         <v>4000</v>
@@ -893,7 +847,7 @@
         <v>4000</v>
       </c>
       <c r="F10" s="4">
-        <v>520</v>
+        <v>786</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -901,10 +855,10 @@
         <v>13</v>
       </c>
       <c r="B11" s="4">
-        <v>48337</v>
+        <v>49006</v>
       </c>
       <c r="C11" s="4">
-        <v>8337</v>
+        <v>9006</v>
       </c>
       <c r="D11" s="4">
         <v>4000</v>
@@ -913,7 +867,7 @@
         <v>4000</v>
       </c>
       <c r="F11" s="4">
-        <v>337</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -921,19 +875,19 @@
         <v>14</v>
       </c>
       <c r="B12" s="4">
-        <v>47878</v>
+        <v>48946</v>
       </c>
       <c r="C12" s="4">
-        <v>7878</v>
+        <v>8946</v>
       </c>
       <c r="D12" s="4">
         <v>4000</v>
       </c>
       <c r="E12" s="4">
-        <v>3878</v>
+        <v>4000</v>
       </c>
       <c r="F12" s="4">
-        <v>0</v>
+        <v>946</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -941,19 +895,19 @@
         <v>15</v>
       </c>
       <c r="B13" s="4">
-        <v>47342</v>
+        <v>48689</v>
       </c>
       <c r="C13" s="4">
-        <v>7342</v>
+        <v>8689</v>
       </c>
       <c r="D13" s="4">
         <v>4000</v>
       </c>
       <c r="E13" s="4">
-        <v>3342</v>
+        <v>4000</v>
       </c>
       <c r="F13" s="4">
-        <v>0</v>
+        <v>689</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1007,10 +961,10 @@
         <v>24000</v>
       </c>
       <c r="D17" s="4">
-        <v>23219</v>
+        <v>24000</v>
       </c>
       <c r="E17" s="5">
-        <v>0.9674672378622982</v>
+        <v>1</v>
       </c>
       <c r="F17" t="s">
         <v>23</v>
@@ -1027,10 +981,10 @@
         <v>24000</v>
       </c>
       <c r="D18" s="4">
-        <v>2353</v>
+        <v>4263</v>
       </c>
       <c r="E18" s="5">
-        <v>0.09804002902803677</v>
+        <v>0.1776442393571094</v>
       </c>
       <c r="F18" t="s">
         <v>26</v>
@@ -1169,22 +1123,22 @@
         <v>43</v>
       </c>
       <c r="C5" s="4">
-        <v>6813</v>
+        <v>6911</v>
       </c>
       <c r="D5" s="4">
-        <v>2737</v>
+        <v>2608</v>
       </c>
       <c r="E5" s="4">
-        <v>6447</v>
+        <v>6559</v>
       </c>
       <c r="F5" s="4">
-        <v>5897</v>
+        <v>5823</v>
       </c>
       <c r="G5" s="4">
-        <v>549</v>
+        <v>735</v>
       </c>
       <c r="H5" s="7">
-        <v>0.125</v>
+        <v>0.142</v>
       </c>
       <c r="I5" s="4">
         <v>0</v>
@@ -1198,25 +1152,25 @@
         <v>45</v>
       </c>
       <c r="C6" s="4">
-        <v>7822</v>
+        <v>8357</v>
       </c>
       <c r="D6" s="4">
-        <v>3186</v>
+        <v>2686</v>
       </c>
       <c r="E6" s="4">
-        <v>8371</v>
+        <v>8170</v>
       </c>
       <c r="F6" s="4">
-        <v>3053</v>
+        <v>2910</v>
       </c>
       <c r="G6" s="4">
-        <v>5318</v>
+        <v>5260</v>
       </c>
       <c r="H6" s="7">
-        <v>0.141</v>
+        <v>0.147</v>
       </c>
       <c r="I6" s="4">
-        <v>3323</v>
+        <v>3409</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1227,25 +1181,25 @@
         <v>47</v>
       </c>
       <c r="C7" s="4">
-        <v>7102</v>
+        <v>7431</v>
       </c>
       <c r="D7" s="4">
-        <v>2377</v>
+        <v>2319</v>
       </c>
       <c r="E7" s="4">
-        <v>6953</v>
+        <v>7359</v>
       </c>
       <c r="F7" s="4">
-        <v>2743</v>
+        <v>2556</v>
       </c>
       <c r="G7" s="4">
-        <v>4210</v>
+        <v>4803</v>
       </c>
       <c r="H7" s="7">
-        <v>0.192</v>
+        <v>0.137</v>
       </c>
       <c r="I7" s="4">
-        <v>2100</v>
+        <v>3372</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1256,25 +1210,25 @@
         <v>49</v>
       </c>
       <c r="C8" s="4">
-        <v>4695</v>
+        <v>4933</v>
       </c>
       <c r="D8" s="4">
-        <v>2344</v>
+        <v>2487</v>
       </c>
       <c r="E8" s="4">
-        <v>5106</v>
+        <v>5138</v>
       </c>
       <c r="F8" s="4">
-        <v>1861</v>
+        <v>1710</v>
       </c>
       <c r="G8" s="4">
-        <v>3245</v>
+        <v>3428</v>
       </c>
       <c r="H8" s="7">
-        <v>0.134</v>
+        <v>0.156</v>
       </c>
       <c r="I8" s="4">
-        <v>1703</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1285,22 +1239,22 @@
         <v>51</v>
       </c>
       <c r="C9" s="4">
-        <v>2913</v>
+        <v>2867</v>
       </c>
       <c r="D9" s="4">
-        <v>2067</v>
+        <v>1917</v>
       </c>
       <c r="E9" s="4">
-        <v>3020</v>
+        <v>2930</v>
       </c>
       <c r="F9" s="4">
-        <v>2698</v>
+        <v>2616</v>
       </c>
       <c r="G9" s="4">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="H9" s="7">
-        <v>0.079</v>
+        <v>0.091</v>
       </c>
       <c r="I9" s="4">
         <v>0</v>
@@ -1314,22 +1268,22 @@
         <v>53</v>
       </c>
       <c r="C10" s="4">
-        <v>2085</v>
+        <v>2096</v>
       </c>
       <c r="D10" s="4">
-        <v>1351</v>
+        <v>1387</v>
       </c>
       <c r="E10" s="4">
-        <v>2143</v>
+        <v>2086</v>
       </c>
       <c r="F10" s="4">
-        <v>1997</v>
+        <v>2007</v>
       </c>
       <c r="G10" s="4">
-        <v>146</v>
+        <v>79</v>
       </c>
       <c r="H10" s="7">
-        <v>0.096</v>
+        <v>0.119</v>
       </c>
       <c r="I10" s="4">
         <v>0</v>
@@ -1343,22 +1297,22 @@
         <v>55</v>
       </c>
       <c r="C11" s="4">
-        <v>2998</v>
+        <v>2919</v>
       </c>
       <c r="D11" s="4">
-        <v>1485</v>
+        <v>1456</v>
       </c>
       <c r="E11" s="4">
-        <v>2912</v>
+        <v>2831</v>
       </c>
       <c r="F11" s="4">
-        <v>2515</v>
+        <v>2535</v>
       </c>
       <c r="G11" s="4">
-        <v>396</v>
+        <v>295</v>
       </c>
       <c r="H11" s="7">
-        <v>0.073</v>
+        <v>0.125</v>
       </c>
       <c r="I11" s="4">
         <v>0</v>
@@ -1372,22 +1326,22 @@
         <v>57</v>
       </c>
       <c r="C12" s="4">
-        <v>2352</v>
+        <v>2412</v>
       </c>
       <c r="D12" s="4">
-        <v>1130</v>
+        <v>935</v>
       </c>
       <c r="E12" s="4">
-        <v>2405</v>
+        <v>2199</v>
       </c>
       <c r="F12" s="4">
-        <v>2316</v>
+        <v>2363</v>
       </c>
       <c r="G12" s="4">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H12" s="7">
-        <v>0.183</v>
+        <v>0.165</v>
       </c>
       <c r="I12" s="4">
         <v>0</v>
@@ -1401,22 +1355,22 @@
         <v>59</v>
       </c>
       <c r="C13" s="4">
-        <v>1608</v>
+        <v>1622</v>
       </c>
       <c r="D13" s="4">
-        <v>1569</v>
+        <v>1437</v>
       </c>
       <c r="E13" s="4">
-        <v>1756</v>
+        <v>1470</v>
       </c>
       <c r="F13" s="4">
-        <v>1536</v>
+        <v>1550</v>
       </c>
       <c r="G13" s="4">
-        <v>220</v>
+        <v>0</v>
       </c>
       <c r="H13" s="7">
-        <v>0.062</v>
+        <v>0.107</v>
       </c>
       <c r="I13" s="4">
         <v>0</v>
@@ -1430,22 +1384,22 @@
         <v>61</v>
       </c>
       <c r="C14" s="4">
-        <v>2208</v>
+        <v>2213</v>
       </c>
       <c r="D14" s="4">
-        <v>1347</v>
+        <v>1287</v>
       </c>
       <c r="E14" s="4">
-        <v>2318</v>
+        <v>2238</v>
       </c>
       <c r="F14" s="4">
-        <v>2035</v>
+        <v>2111</v>
       </c>
       <c r="G14" s="4">
-        <v>283</v>
+        <v>126</v>
       </c>
       <c r="H14" s="7">
-        <v>0.095</v>
+        <v>0.114</v>
       </c>
       <c r="I14" s="4">
         <v>0</v>
@@ -1459,25 +1413,25 @@
         <v>63</v>
       </c>
       <c r="C15" s="4">
-        <v>3216</v>
+        <v>3341</v>
       </c>
       <c r="D15" s="4">
-        <v>314</v>
+        <v>253</v>
       </c>
       <c r="E15" s="4">
-        <v>2925</v>
+        <v>2986</v>
       </c>
       <c r="F15" s="4">
-        <v>686</v>
+        <v>660</v>
       </c>
       <c r="G15" s="4">
-        <v>2239</v>
+        <v>2326</v>
       </c>
       <c r="H15" s="7">
-        <v>0.238</v>
+        <v>0.209</v>
       </c>
       <c r="I15" s="4">
-        <v>1728</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1488,25 +1442,25 @@
         <v>65</v>
       </c>
       <c r="C16" s="4">
-        <v>3736</v>
+        <v>4090</v>
       </c>
       <c r="D16" s="4">
-        <v>1680</v>
+        <v>1439</v>
       </c>
       <c r="E16" s="4">
-        <v>3988</v>
+        <v>4014</v>
       </c>
       <c r="F16" s="4">
-        <v>1459</v>
+        <v>1321</v>
       </c>
       <c r="G16" s="4">
-        <v>2529</v>
+        <v>2694</v>
       </c>
       <c r="H16" s="7">
-        <v>0.162</v>
+        <v>0.192</v>
       </c>
       <c r="I16" s="4">
-        <v>1269</v>
+        <v>1413</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1517,22 +1471,22 @@
         <v>67</v>
       </c>
       <c r="C17" s="4">
-        <v>1878</v>
+        <v>1920</v>
       </c>
       <c r="D17" s="4">
-        <v>1169</v>
+        <v>1083</v>
       </c>
       <c r="E17" s="4">
-        <v>2082</v>
+        <v>1972</v>
       </c>
       <c r="F17" s="4">
-        <v>1800</v>
+        <v>1939</v>
       </c>
       <c r="G17" s="4">
-        <v>282</v>
+        <v>33</v>
       </c>
       <c r="H17" s="7">
-        <v>0.106</v>
+        <v>0.214</v>
       </c>
       <c r="I17" s="4">
         <v>0</v>
@@ -1546,22 +1500,22 @@
         <v>69</v>
       </c>
       <c r="C18" s="4">
-        <v>1023</v>
+        <v>1068</v>
       </c>
       <c r="D18" s="4">
-        <v>949</v>
+        <v>875</v>
       </c>
       <c r="E18" s="4">
-        <v>1245</v>
+        <v>1121</v>
       </c>
       <c r="F18" s="4">
-        <v>1011</v>
+        <v>1048</v>
       </c>
       <c r="G18" s="4">
-        <v>234</v>
+        <v>74</v>
       </c>
       <c r="H18" s="7">
-        <v>0.154</v>
+        <v>0.126</v>
       </c>
       <c r="I18" s="4">
         <v>0</v>
@@ -1573,23 +1527,23 @@
         <v>70</v>
       </c>
       <c r="C19" s="9">
-        <v>50449</v>
+        <v>52180</v>
       </c>
       <c r="D19" s="9">
-        <v>23705</v>
+        <v>22169</v>
       </c>
       <c r="E19" s="9">
-        <v>51671</v>
+        <v>51073</v>
       </c>
       <c r="F19" s="9">
-        <v>31607</v>
+        <v>31149</v>
       </c>
       <c r="G19" s="9">
-        <v>20063</v>
+        <v>20166</v>
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="9">
-        <v>10123</v>
+        <v>11826</v>
       </c>
     </row>
   </sheetData>
@@ -1598,118 +1552,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5AFCEE-CBE5-5B48-8162-37F5E7CD7B22}">
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" s="4">
-        <v>14929</v>
-      </c>
-      <c r="D5" s="4">
-        <v>13114</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1815</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" s="4">
-        <v>13113</v>
-      </c>
-      <c r="D6" s="4">
-        <v>11524</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1589</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B7" t="s">
-        <v>83</v>
-      </c>
-      <c r="C7" s="4">
-        <v>9387</v>
-      </c>
-      <c r="D7" s="4">
-        <v>8345</v>
-      </c>
-      <c r="E7" s="4">
-        <v>1042</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C8" s="4">
-        <v>7532</v>
-      </c>
-      <c r="D8" s="4">
-        <v>6756</v>
-      </c>
-      <c r="E8" s="4">
-        <v>776</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{733AA36E-D814-5684-BBAA-CB6036F11663}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1723,12 +1565,12 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1736,186 +1578,186 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B5" s="4">
-        <v>1896</v>
+        <v>1801</v>
       </c>
       <c r="C5" s="4">
         <v>458975</v>
       </c>
       <c r="D5" s="4">
-        <v>395449</v>
+        <v>394969</v>
       </c>
       <c r="E5" s="7">
-        <v>0.222</v>
+        <v>0.211</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B6" s="4">
-        <v>2227</v>
+        <v>2181</v>
       </c>
       <c r="C6" s="4">
         <v>399486</v>
       </c>
       <c r="D6" s="4">
-        <v>348266</v>
+        <v>347903</v>
       </c>
       <c r="E6" s="7">
-        <v>0.298</v>
+        <v>0.292</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="B7" s="4">
-        <v>2460</v>
+        <v>2387</v>
       </c>
       <c r="C7" s="4">
         <v>443336</v>
       </c>
       <c r="D7" s="4">
-        <v>404332</v>
+        <v>403357</v>
       </c>
       <c r="E7" s="7">
-        <v>0.29</v>
+        <v>0.282</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B8" s="4">
-        <v>2406</v>
+        <v>2367</v>
       </c>
       <c r="C8" s="4">
         <v>449556</v>
       </c>
       <c r="D8" s="4">
-        <v>395065</v>
+        <v>393209</v>
       </c>
       <c r="E8" s="7">
-        <v>0.285</v>
+        <v>0.281</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="B9" s="4">
-        <v>2499</v>
+        <v>2441</v>
       </c>
       <c r="C9" s="4">
         <v>471224</v>
       </c>
       <c r="D9" s="4">
-        <v>424606</v>
+        <v>425713</v>
       </c>
       <c r="E9" s="7">
-        <v>0.279</v>
+        <v>0.272</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="B10" s="4">
-        <v>2653</v>
+        <v>2602</v>
       </c>
       <c r="C10" s="4">
         <v>483430</v>
       </c>
       <c r="D10" s="4">
-        <v>435139</v>
+        <v>435913</v>
       </c>
       <c r="E10" s="7">
-        <v>0.289</v>
+        <v>0.283</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="B11" s="4">
-        <v>2829</v>
+        <v>2919</v>
       </c>
       <c r="C11" s="4">
         <v>515466</v>
       </c>
       <c r="D11" s="4">
-        <v>457363</v>
+        <v>454441</v>
       </c>
       <c r="E11" s="7">
-        <v>0.291</v>
+        <v>0.301</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>84</v>
       </c>
       <c r="B12" s="4">
-        <v>3039</v>
+        <v>3151</v>
       </c>
       <c r="C12" s="4">
         <v>511283</v>
       </c>
       <c r="D12" s="4">
-        <v>465221</v>
+        <v>464810</v>
       </c>
       <c r="E12" s="7">
-        <v>0.311</v>
+        <v>0.323</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
       <c r="B13" s="4">
-        <v>3434</v>
+        <v>3612</v>
       </c>
       <c r="C13" s="4">
         <v>518010</v>
       </c>
       <c r="D13" s="4">
-        <v>474147</v>
+        <v>473848</v>
       </c>
       <c r="E13" s="7">
-        <v>0.346</v>
+        <v>0.364</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="B14" s="4">
-        <v>3356</v>
+        <v>3603</v>
       </c>
       <c r="C14" s="4">
         <v>536610</v>
       </c>
       <c r="D14" s="4">
-        <v>486089</v>
+        <v>486459</v>
       </c>
       <c r="E14" s="7">
-        <v>0.328</v>
+        <v>0.352</v>
       </c>
     </row>
   </sheetData>
@@ -1923,7 +1765,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C55AA092-8E7A-548F-8863-3CB3460A96CF}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1934,87 +1776,87 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>106</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>112</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>114</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>